<commit_message>
Guia de videos para reporte y registro
Se aclara y actualiza la inforamción en el dashboard
</commit_message>
<xml_diff>
--- a/Datos_Malla_SALVIA.xlsx
+++ b/Datos_Malla_SALVIA.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2417" uniqueCount="1056">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2423" uniqueCount="1060">
   <si>
     <t xml:space="preserve">Malla SALVIA Etapa 2</t>
   </si>
@@ -633,7 +633,7 @@
     <t xml:space="preserve">Mockup navegable y guia de videos</t>
   </si>
   <si>
-    <t xml:space="preserve">Mockup y guía de 22 videos entregados el 27-sep</t>
+    <t xml:space="preserve">Mockup y guía de 22 videos entregados el 27-sep; los videos no se grabaron porque el HTML pasó directo al equipo de desarrollo</t>
   </si>
   <si>
     <t xml:space="preserve">4.4.3</t>
@@ -990,7 +990,7 @@
     <t xml:space="preserve">Reporte y Registro operativos</t>
   </si>
   <si>
-    <t xml:space="preserve">Lista para main (corte 13-oct): nueva versión del formulario público de reporte ciudadano. Segunda versión del reporte ciudadano construida el 27-sep (PSWYA-755), sin llegar a main; el nuevo Registro no tiene desarrollo</t>
+    <t xml:space="preserve">El HTML del mockup y sus componentes se entregaron al equipo de desarrollo para pasarlos al servidor de pruebas, entrega prevista para finales de la semana del 13-oct o, a más tardar, a mediados de la semana del 20-oct. Antes: Lista para main (corte 13-oct): nueva versión del formulario público de reporte ciudadano. Segunda versión del reporte ciudadano construida el 27-sep (PSWYA-755), sin llegar a main; el nuevo Registro no tiene desarrollo</t>
   </si>
   <si>
     <t xml:space="preserve">6.1.9</t>
@@ -1803,7 +1803,7 @@
     <t xml:space="preserve">M2 · TAMIZAJE DE FEMINICIDIO</t>
   </si>
   <si>
-    <t xml:space="preserve">Avance: Gestión del Conocimiento aprobó el mockup de Reportes, Registro y Alerta Inminente (según el equipo, 13-oct), que incluye el formulario completo del tamizaje de feminicidio con bifurcaciones OSIGD y pareja/no pareja, puntaje y alertas por nivel de riesgo. En producción operan la parametrización de tiempos, la clasificación alto/bajo y la asignación automática. Pendiente: confirmar los rangos del puntaje y construir el nuevo formulario de registro. Nota: el trabajo del mockup no aparece completo en las horas reportadas; se registra como evidencia en la hoja Trabajo_sin_horas.</t>
+    <t xml:space="preserve">Avance: Gestión del Conocimiento aprobó el mockup de Reportes, Registro y Alerta Inminente (según el equipo, 13-oct), que incluye el formulario completo del tamizaje de feminicidio con bifurcaciones OSIGD y pareja/no pareja, puntaje y alertas por nivel de riesgo. En producción operan la parametrización de tiempos, la clasificación alto/bajo y la asignación automática. Pendiente: confirmar los rangos del puntaje; el HTML del mockup ya está con el equipo de desarrollo y su paso al servidor de pruebas está prevista para finales de la semana del 13-oct o, a más tardar, a mediados de la semana del 20-oct. Nota: el trabajo del mockup no aparece completo en las horas reportadas; se registra como evidencia en la hoja Trabajo_sin_horas.</t>
   </si>
   <si>
     <t xml:space="preserve">Brayan Marbello</t>
@@ -1821,13 +1821,13 @@
     <t xml:space="preserve">M4 · LGBTIQ+</t>
   </si>
   <si>
-    <t xml:space="preserve">Avance: el mockup aprobado de Reportes, Registro y Alerta Inminente incluye las preguntas OSIGD y el tamizaje diferencial para población LGBTIQ+ dentro del mismo formulario, sin módulo aparte; secciones OSIGHN construidas en psicosocial el 17-sep. Pendiente: construir el MVP en registro y seguimiento. Riesgo: la pregunta OSIGHN aparece hoy donde no corresponde (hallazgo PSI-24). Nota: el trabajo del mockup se registra como evidencia en la hoja Trabajo_sin_horas, sin sumar horas.</t>
+    <t xml:space="preserve">Avance: el mockup aprobado de Reportes, Registro y Alerta Inminente incluye las preguntas OSIGD y el tamizaje diferencial para población LGBTIQ+ dentro del mismo formulario, sin módulo aparte; secciones OSIGHN construidas en psicosocial el 17-sep. Pendiente: construir el MVP en registro y seguimiento; el HTML del mockup ya está con el equipo de desarrollo y su paso al servidor de pruebas está prevista para finales de la semana del 13-oct o, a más tardar, a mediados de la semana del 20-oct. Riesgo: la pregunta OSIGHN aparece hoy donde no corresponde (hallazgo PSI-24). Nota: el trabajo del mockup se registra como evidencia en la hoja Trabajo_sin_horas, sin sumar horas.</t>
   </si>
   <si>
     <t xml:space="preserve">M5 · ASP (MODULO WEB)</t>
   </si>
   <si>
-    <t xml:space="preserve">Avance: el mockup aprobado de Reportes, Registro y Alerta Inminente incluye el formulario del módulo web ASP dentro del registro de la víctima. Pendiente: construcción del módulo web. Decisión: la solicitud de prórroga del 22-sep pide a la Supervisión definir el tratamiento del desarrollo integral del módulo y su app. Riesgo: los lineamientos de la Dirección de Actividades Sexuales Pagas no se han recibido formalmente. Nota: el trabajo del mockup se registra como evidencia en la hoja Trabajo_sin_horas, sin sumar horas.</t>
+    <t xml:space="preserve">Avance: el mockup aprobado de Reportes, Registro y Alerta Inminente incluye el formulario del módulo web ASP dentro del registro de la víctima. Pendiente: construcción del módulo web; el formulario de registro ya está con el equipo de desarrollo para pasar al servidor de pruebas. Decisión: la solicitud de prórroga del 22-sep pide a la Supervisión definir el tratamiento del desarrollo integral del módulo y su app. Riesgo: los lineamientos de la Dirección de Actividades Sexuales Pagas no se han recibido formalmente. Nota: el trabajo del mockup se registra como evidencia en la hoja Trabajo_sin_horas, sin sumar horas.</t>
   </si>
   <si>
     <t xml:space="preserve">Santiago Ramos / Juan Buitrago</t>
@@ -2077,7 +2077,7 @@
     <t xml:space="preserve">Oct 2026 · corte 13-oct</t>
   </si>
   <si>
-    <t xml:space="preserve">Gestión del Conocimiento aprobó el mockup de Reportes, Registro y Alerta Inminente, que incluye los formularios de tamizaje, LGBTIQ+ y ASP.
+    <t xml:space="preserve">Gestión del Conocimiento aprobó el mockup de Reportes, Registro y Alerta Inminente, que incluye los formularios de tamizaje, LGBTIQ+ y ASP; el HTML ya está con el equipo de desarrollo y su paso al servidor de pruebas está prevista para finales de la semana del 13-oct o, a más tardar, a mediados de la semana del 20-oct.
 64 cambios listos para el próximo despliegue a main (corte 13-oct), varios de ellos hallazgos que el equipo no había reportado como resueltos.
 La matriz de hallazgos de SALVIA da por cerrados 107 de 159 (revisión Kreivo del 8-oct).
 Solicitud de prórroga hasta el 15-dic radicada el 22-sep, pendiente de decisión.
@@ -3200,16 +3200,28 @@
     <t xml:space="preserve">38 historias en 12 grupos: remisión, riesgo inminente, revisión del Equipo Técnico, bandeja y asignación, consentimiento y caracterización, aprobación, Cruz Roja, seguimiento, matriz de medidas, novedades, conclusión y trazabilidad. No cubren familiares ni personas huérfanas.</t>
   </si>
   <si>
-    <t xml:space="preserve">Guía de videos del mockup de Reporte y Registro (22 partes)</t>
+    <t xml:space="preserve">Guía y guion de grabación de los 22 videos del mockup de Reporte y Registro</t>
   </si>
   <si>
     <t xml:space="preserve">Documentación</t>
   </si>
   <si>
-    <t xml:space="preserve">Entregada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recorrido del mockup y los 10 puntos que se tomaron donde el guion y el formulario no coincidían.</t>
+    <t xml:space="preserve">Entregados; los videos no se grabaron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guía funcional de las 22 partes y guion de grabación clip a clip. Los videos no se grabaron porque el HTML y sus componentes se entregaron directamente al equipo de desarrollo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega del HTML del mockup de Reporte y Registro al equipo de desarrollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desarrollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En construcción; paso al servidor de pruebas prevista para finales de la semana del 13-oct o, a más tardar, a mediados de la semana del 20-oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El equipo de desarrollo toma el HTML y sus componentes para construir el nuevo Reporte y Registro (formularios de tamizaje, LGBTIQ+ y ASP) en el servidor de pruebas.</t>
   </si>
   <si>
     <t xml:space="preserve">64 cambios listos para el próximo despliegue a main</t>
@@ -6723,7 +6735,7 @@
       </c>
       <c r="K54" s="19" t="n">
         <f aca="false">Plan!E73</f>
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="L54" s="16" t="s">
         <v>873</v>
@@ -10281,7 +10293,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -10408,7 +10420,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="n">
         <v>46308</v>
       </c>
@@ -10419,21 +10431,44 @@
         <v>1050</v>
       </c>
       <c r="D6" s="17" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="F6" s="17" t="s">
         <v>1051</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="G6" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="F6" s="17" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>1053</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="C7" s="17" t="s">
         <v>1054</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="D7" s="17" t="s">
         <v>1055</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>1057</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>
@@ -12571,7 +12606,7 @@
       </c>
       <c r="E64" s="6" t="n">
         <f aca="false">SUMPRODUCT((D65:D85=3)*E65:E85)/COUNTIF(D65:D85,3)</f>
-        <v>0.421052631578947</v>
+        <v>0.423684210526316</v>
       </c>
       <c r="F64" s="2" t="str">
         <f aca="false">IF(E64&gt;=0.995,"Completado",IF(E64&gt;0,"En curso","Pendiente"))</f>
@@ -12602,7 +12637,7 @@
       </c>
       <c r="E65" s="6" t="n">
         <f aca="false">SUMPRODUCT((D66:D77=3)*E66:E77)/COUNTIF(D66:D77,3)</f>
-        <v>0.429166666666667</v>
+        <v>0.433333333333333</v>
       </c>
       <c r="F65" s="2" t="str">
         <f aca="false">IF(E65&gt;=0.995,"Completado",IF(E65&gt;0,"En curso","Pendiente"))</f>
@@ -12856,7 +12891,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
         <v>314</v>
       </c>
@@ -12870,7 +12905,7 @@
         <v>3</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="F73" s="1" t="str">
         <f aca="false">IF(E73&gt;=0.995,"Completado",IF(E73&gt;0,"En curso","Pendiente"))</f>
@@ -12880,7 +12915,7 @@
         <v>317</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="I73" s="1" t="n">
         <f aca="false">IF(E73&gt;=0.995,3,IF(E73&gt;0,2,1))</f>
@@ -23109,7 +23144,7 @@
       </c>
       <c r="D3" s="13" t="n">
         <f aca="false">SUMPRODUCT((Pertenencia!C$2:C$145=1)*(Plan!$D$2:$D$145=3)*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!C$2:C$145=1)*(Plan!$D$2:$D$145=3))</f>
-        <v>0.736363636363636</v>
+        <v>0.740909090909091</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>588</v>
@@ -23129,7 +23164,7 @@
       </c>
       <c r="J3" s="13" t="n">
         <f aca="false">IF(SUMPRODUCT((Pertenencia!C$2:C$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre"))=0,"",SUMPRODUCT((Pertenencia!C$2:C$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!C$2:C$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")))</f>
-        <v>0.483333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>586</v>
@@ -23183,7 +23218,7 @@
       </c>
       <c r="D5" s="13" t="n">
         <f aca="false">SUMPRODUCT((Pertenencia!E$2:E$145=1)*(Plan!$D$2:$D$145=3)*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!E$2:E$145=1)*(Plan!$D$2:$D$145=3))</f>
-        <v>0.75</v>
+        <v>0.75625</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>594</v>
@@ -23203,7 +23238,7 @@
       </c>
       <c r="J5" s="13" t="n">
         <f aca="false">IF(SUMPRODUCT((Pertenencia!E$2:E$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre"))=0,"",SUMPRODUCT((Pertenencia!E$2:E$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!E$2:E$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")))</f>
-        <v>0.3</v>
+        <v>0.325</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>586</v>
@@ -23221,7 +23256,7 @@
       </c>
       <c r="D6" s="13" t="n">
         <f aca="false">SUMPRODUCT((Pertenencia!F$2:F$145=1)*(Plan!$D$2:$D$145=3)*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!F$2:F$145=1)*(Plan!$D$2:$D$145=3))</f>
-        <v>0.622222222222222</v>
+        <v>0.627777777777778</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>596</v>
@@ -23241,7 +23276,7 @@
       </c>
       <c r="J6" s="13" t="n">
         <f aca="false">IF(SUMPRODUCT((Pertenencia!F$2:F$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre"))=0,"",SUMPRODUCT((Pertenencia!F$2:F$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")*Plan!$E$2:$E$145)/SUMPRODUCT((Pertenencia!F$2:F$145=1)*(Plan!$D$2:$D$145=3)*(Plan!$J$2:$J$145="Construcción y cierre")))</f>
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>586</v>
@@ -29917,7 +29952,7 @@
       </c>
       <c r="F9" s="17"/>
     </row>
-    <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
         <v>670</v>
       </c>
@@ -31324,13 +31359,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B568A7-566D-403B-8645-C34DDB677C9A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6491DF5-1C94-473E-A2CC-940B67F7F853}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C27CA390-DE3F-41D0-81D9-3BF35A4ADEDD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{529CBF12-9307-494A-A0C4-F5F6681D5C7E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7F27B64-AF70-405F-ACBF-18DC41833E71}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BE0B505-4775-49EE-AA01-998A89548AED}"/>
 </file>
</xml_diff>